<commit_message>
Improve cost templates and donut interaction
</commit_message>
<xml_diff>
--- a/public/templates/tts-cost-inputs.xlsx
+++ b/public/templates/tts-cost-inputs.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Cost" sheetId="1" r:id="R67fe49bc0f364b63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agency Fee Rules" sheetId="2" r:id="Rbf0c9c44045e4bd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Return Shipping Cost" sheetId="3" r:id="Rea55fc979a0c409d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual Costs" sheetId="4" r:id="R03e3247e6e6b488d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Cost" sheetId="1" r:id="Rdcd174d7332c4e1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agency Fee Rules" sheetId="2" r:id="Re0f57d39521549d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Return Shipping Cost" sheetId="3" r:id="R71bd5784d9614da9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual Costs" sheetId="4" r:id="R3fa6bf9925444305"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,11 +16,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="4">
+  <x:numFmts count="5">
     <x:numFmt numFmtId="200" formatCode="$#,##0.00"/>
     <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="202" formatCode="0.00%;[Red](0.00%)"/>
     <x:numFmt numFmtId="203" formatCode="$#,##0.00;[Red]($#,##0.00);-"/>
+    <x:numFmt numFmtId="204" formatCode="@"/>
   </x:numFmts>
   <x:fonts count="6">
     <x:font>
@@ -144,7 +145,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="31">
+  <x:cellXfs count="33">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -188,6 +189,8 @@
     <x:xf numFmtId="203" fontId="0" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="4" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="0" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -434,410 +437,480 @@
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="19" t="str">
-        <x:v>ASP-BLUE</x:v>
-      </x:c>
-      <x:c r="B7" s="19" t="str">
-        <x:v>Airstyle Pro Blue</x:v>
-      </x:c>
-      <x:c r="C7" s="21" t="n">
-        <x:v>62</x:v>
-      </x:c>
+      <x:c r="A7" s="31" t="str">
+        <x:v>Chrona_BG</x:v>
+      </x:c>
+      <x:c r="B7" s="31" t="str">
+        <x:v>Chrona_BG</x:v>
+      </x:c>
+      <x:c r="C7" s="21"/>
       <x:c r="D7" s="23" t="n">
-        <x:v>46235</x:v>
+        <x:v>46143</x:v>
       </x:c>
       <x:c r="E7" s="23"/>
       <x:c r="F7" s="19" t="str">
-        <x:v>Current Cost</x:v>
+        <x:v>Enter unit cost</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="20"/>
-      <x:c r="B8" s="20"/>
+      <x:c r="A8" s="32" t="str">
+        <x:v>Pocket_Pro</x:v>
+      </x:c>
+      <x:c r="B8" s="32" t="str">
+        <x:v>Pocket_Pro</x:v>
+      </x:c>
       <x:c r="C8" s="22"/>
-      <x:c r="D8" s="24"/>
+      <x:c r="D8" s="24" t="n">
+        <x:v>46143</x:v>
+      </x:c>
       <x:c r="E8" s="24"/>
-      <x:c r="F8" s="20"/>
+      <x:c r="F8" s="20" t="str">
+        <x:v>Enter unit cost</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="20"/>
-      <x:c r="B9" s="20"/>
+      <x:c r="A9" s="32" t="str">
+        <x:v>L10S_Pro_Ultra</x:v>
+      </x:c>
+      <x:c r="B9" s="32" t="str">
+        <x:v>L10S_Pro_Ultra</x:v>
+      </x:c>
       <x:c r="C9" s="22"/>
-      <x:c r="D9" s="24"/>
+      <x:c r="D9" s="24" t="n">
+        <x:v>46143</x:v>
+      </x:c>
       <x:c r="E9" s="24"/>
-      <x:c r="F9" s="20"/>
+      <x:c r="F9" s="20" t="str">
+        <x:v>Enter unit cost</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="20"/>
-      <x:c r="B10" s="20"/>
+      <x:c r="A10" s="32" t="str">
+        <x:v>Pocket_Pure</x:v>
+      </x:c>
+      <x:c r="B10" s="32" t="str">
+        <x:v>Pocket_Pure</x:v>
+      </x:c>
       <x:c r="C10" s="22"/>
-      <x:c r="D10" s="24"/>
+      <x:c r="D10" s="24" t="n">
+        <x:v>46143</x:v>
+      </x:c>
       <x:c r="E10" s="24"/>
-      <x:c r="F10" s="20"/>
+      <x:c r="F10" s="20" t="str">
+        <x:v>Enter unit cost</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="20"/>
-      <x:c r="B11" s="20"/>
+      <x:c r="A11" s="32" t="str">
+        <x:v>Glory_Combo</x:v>
+      </x:c>
+      <x:c r="B11" s="32" t="str">
+        <x:v>Glory_Combo</x:v>
+      </x:c>
       <x:c r="C11" s="22"/>
-      <x:c r="D11" s="24"/>
+      <x:c r="D11" s="24" t="n">
+        <x:v>46143</x:v>
+      </x:c>
       <x:c r="E11" s="24"/>
-      <x:c r="F11" s="20"/>
+      <x:c r="F11" s="20" t="str">
+        <x:v>Enter unit cost</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="20"/>
-      <x:c r="B12" s="20"/>
+      <x:c r="A12" s="32" t="str">
+        <x:v>Airstyle_Suite</x:v>
+      </x:c>
+      <x:c r="B12" s="32" t="str">
+        <x:v>Airstyle_Suite</x:v>
+      </x:c>
       <x:c r="C12" s="22"/>
-      <x:c r="D12" s="24"/>
+      <x:c r="D12" s="24" t="n">
+        <x:v>46143</x:v>
+      </x:c>
       <x:c r="E12" s="24"/>
-      <x:c r="F12" s="20"/>
+      <x:c r="F12" s="20" t="str">
+        <x:v>Enter unit cost</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="20"/>
-      <x:c r="B13" s="20"/>
+      <x:c r="A13" s="32" t="str">
+        <x:v>Airstyle_Era</x:v>
+      </x:c>
+      <x:c r="B13" s="32" t="str">
+        <x:v>Airstyle_Era</x:v>
+      </x:c>
       <x:c r="C13" s="22"/>
-      <x:c r="D13" s="24"/>
+      <x:c r="D13" s="24" t="n">
+        <x:v>46143</x:v>
+      </x:c>
       <x:c r="E13" s="24"/>
-      <x:c r="F13" s="20"/>
+      <x:c r="F13" s="20" t="str">
+        <x:v>Enter unit cost</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="20"/>
-      <x:c r="B14" s="20"/>
+      <x:c r="A14" s="32" t="str">
+        <x:v>Pocket_2026</x:v>
+      </x:c>
+      <x:c r="B14" s="32" t="str">
+        <x:v>Pocket_2026</x:v>
+      </x:c>
       <x:c r="C14" s="22"/>
-      <x:c r="D14" s="24"/>
+      <x:c r="D14" s="24" t="n">
+        <x:v>46143</x:v>
+      </x:c>
       <x:c r="E14" s="24"/>
-      <x:c r="F14" s="20"/>
+      <x:c r="F14" s="20" t="str">
+        <x:v>Enter unit cost</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="20"/>
-      <x:c r="B15" s="20"/>
+      <x:c r="A15" s="32" t="str">
+        <x:v>Airstyle_Pro</x:v>
+      </x:c>
+      <x:c r="B15" s="32" t="str">
+        <x:v>Airstyle_Pro</x:v>
+      </x:c>
       <x:c r="C15" s="22"/>
-      <x:c r="D15" s="24"/>
+      <x:c r="D15" s="24" t="n">
+        <x:v>46143</x:v>
+      </x:c>
       <x:c r="E15" s="24"/>
-      <x:c r="F15" s="20"/>
+      <x:c r="F15" s="20" t="str">
+        <x:v>Enter unit cost</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="20"/>
-      <x:c r="B16" s="20"/>
+      <x:c r="A16" s="32" t="str">
+        <x:v>L10SUltraGen2</x:v>
+      </x:c>
+      <x:c r="B16" s="32" t="str">
+        <x:v>L10SUltraGen2</x:v>
+      </x:c>
       <x:c r="C16" s="22"/>
-      <x:c r="D16" s="24"/>
+      <x:c r="D16" s="24" t="n">
+        <x:v>46143</x:v>
+      </x:c>
       <x:c r="E16" s="24"/>
-      <x:c r="F16" s="20"/>
+      <x:c r="F16" s="20" t="str">
+        <x:v>Enter unit cost</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="20"/>
-      <x:c r="B17" s="20"/>
+      <x:c r="A17" s="32"/>
+      <x:c r="B17" s="32"/>
       <x:c r="C17" s="22"/>
       <x:c r="D17" s="24"/>
       <x:c r="E17" s="24"/>
       <x:c r="F17" s="20"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="20"/>
-      <x:c r="B18" s="20"/>
+      <x:c r="A18" s="32"/>
+      <x:c r="B18" s="32"/>
       <x:c r="C18" s="22"/>
       <x:c r="D18" s="24"/>
       <x:c r="E18" s="24"/>
       <x:c r="F18" s="20"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="20"/>
-      <x:c r="B19" s="20"/>
+      <x:c r="A19" s="32"/>
+      <x:c r="B19" s="32"/>
       <x:c r="C19" s="22"/>
       <x:c r="D19" s="24"/>
       <x:c r="E19" s="24"/>
       <x:c r="F19" s="20"/>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="20"/>
-      <x:c r="B20" s="20"/>
+      <x:c r="A20" s="32"/>
+      <x:c r="B20" s="32"/>
       <x:c r="C20" s="22"/>
       <x:c r="D20" s="24"/>
       <x:c r="E20" s="24"/>
       <x:c r="F20" s="20"/>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="20"/>
-      <x:c r="B21" s="20"/>
+      <x:c r="A21" s="32"/>
+      <x:c r="B21" s="32"/>
       <x:c r="C21" s="22"/>
       <x:c r="D21" s="24"/>
       <x:c r="E21" s="24"/>
       <x:c r="F21" s="20"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="20"/>
-      <x:c r="B22" s="20"/>
+      <x:c r="A22" s="32"/>
+      <x:c r="B22" s="32"/>
       <x:c r="C22" s="22"/>
       <x:c r="D22" s="24"/>
       <x:c r="E22" s="24"/>
       <x:c r="F22" s="20"/>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="20"/>
-      <x:c r="B23" s="20"/>
+      <x:c r="A23" s="32"/>
+      <x:c r="B23" s="32"/>
       <x:c r="C23" s="22"/>
       <x:c r="D23" s="24"/>
       <x:c r="E23" s="24"/>
       <x:c r="F23" s="20"/>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="20"/>
-      <x:c r="B24" s="20"/>
+      <x:c r="A24" s="32"/>
+      <x:c r="B24" s="32"/>
       <x:c r="C24" s="22"/>
       <x:c r="D24" s="24"/>
       <x:c r="E24" s="24"/>
       <x:c r="F24" s="20"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="20"/>
-      <x:c r="B25" s="20"/>
+      <x:c r="A25" s="32"/>
+      <x:c r="B25" s="32"/>
       <x:c r="C25" s="22"/>
       <x:c r="D25" s="24"/>
       <x:c r="E25" s="24"/>
       <x:c r="F25" s="20"/>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="20"/>
-      <x:c r="B26" s="20"/>
+      <x:c r="A26" s="32"/>
+      <x:c r="B26" s="32"/>
       <x:c r="C26" s="22"/>
       <x:c r="D26" s="24"/>
       <x:c r="E26" s="24"/>
       <x:c r="F26" s="20"/>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="20"/>
-      <x:c r="B27" s="20"/>
+      <x:c r="A27" s="32"/>
+      <x:c r="B27" s="32"/>
       <x:c r="C27" s="22"/>
       <x:c r="D27" s="24"/>
       <x:c r="E27" s="24"/>
       <x:c r="F27" s="20"/>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="20"/>
-      <x:c r="B28" s="20"/>
+      <x:c r="A28" s="32"/>
+      <x:c r="B28" s="32"/>
       <x:c r="C28" s="22"/>
       <x:c r="D28" s="24"/>
       <x:c r="E28" s="24"/>
       <x:c r="F28" s="20"/>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="20"/>
-      <x:c r="B29" s="20"/>
+      <x:c r="A29" s="32"/>
+      <x:c r="B29" s="32"/>
       <x:c r="C29" s="22"/>
       <x:c r="D29" s="24"/>
       <x:c r="E29" s="24"/>
       <x:c r="F29" s="20"/>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="20"/>
-      <x:c r="B30" s="20"/>
+      <x:c r="A30" s="32"/>
+      <x:c r="B30" s="32"/>
       <x:c r="C30" s="22"/>
       <x:c r="D30" s="24"/>
       <x:c r="E30" s="24"/>
       <x:c r="F30" s="20"/>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="20"/>
-      <x:c r="B31" s="20"/>
+      <x:c r="A31" s="32"/>
+      <x:c r="B31" s="32"/>
       <x:c r="C31" s="22"/>
       <x:c r="D31" s="24"/>
       <x:c r="E31" s="24"/>
       <x:c r="F31" s="20"/>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="20"/>
-      <x:c r="B32" s="20"/>
+      <x:c r="A32" s="32"/>
+      <x:c r="B32" s="32"/>
       <x:c r="C32" s="22"/>
       <x:c r="D32" s="24"/>
       <x:c r="E32" s="24"/>
       <x:c r="F32" s="20"/>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="20"/>
-      <x:c r="B33" s="20"/>
+      <x:c r="A33" s="32"/>
+      <x:c r="B33" s="32"/>
       <x:c r="C33" s="22"/>
       <x:c r="D33" s="24"/>
       <x:c r="E33" s="24"/>
       <x:c r="F33" s="20"/>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="20"/>
-      <x:c r="B34" s="20"/>
+      <x:c r="A34" s="32"/>
+      <x:c r="B34" s="32"/>
       <x:c r="C34" s="22"/>
       <x:c r="D34" s="24"/>
       <x:c r="E34" s="24"/>
       <x:c r="F34" s="20"/>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="20"/>
-      <x:c r="B35" s="20"/>
+      <x:c r="A35" s="32"/>
+      <x:c r="B35" s="32"/>
       <x:c r="C35" s="22"/>
       <x:c r="D35" s="24"/>
       <x:c r="E35" s="24"/>
       <x:c r="F35" s="20"/>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="20"/>
-      <x:c r="B36" s="20"/>
+      <x:c r="A36" s="32"/>
+      <x:c r="B36" s="32"/>
       <x:c r="C36" s="22"/>
       <x:c r="D36" s="24"/>
       <x:c r="E36" s="24"/>
       <x:c r="F36" s="20"/>
     </x:row>
     <x:row r="37">
-      <x:c r="A37" s="20"/>
-      <x:c r="B37" s="20"/>
+      <x:c r="A37" s="32"/>
+      <x:c r="B37" s="32"/>
       <x:c r="C37" s="22"/>
       <x:c r="D37" s="24"/>
       <x:c r="E37" s="24"/>
       <x:c r="F37" s="20"/>
     </x:row>
     <x:row r="38">
-      <x:c r="A38" s="20"/>
-      <x:c r="B38" s="20"/>
+      <x:c r="A38" s="32"/>
+      <x:c r="B38" s="32"/>
       <x:c r="C38" s="22"/>
       <x:c r="D38" s="24"/>
       <x:c r="E38" s="24"/>
       <x:c r="F38" s="20"/>
     </x:row>
     <x:row r="39">
-      <x:c r="A39" s="20"/>
-      <x:c r="B39" s="20"/>
+      <x:c r="A39" s="32"/>
+      <x:c r="B39" s="32"/>
       <x:c r="C39" s="22"/>
       <x:c r="D39" s="24"/>
       <x:c r="E39" s="24"/>
       <x:c r="F39" s="20"/>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="20"/>
-      <x:c r="B40" s="20"/>
+      <x:c r="A40" s="32"/>
+      <x:c r="B40" s="32"/>
       <x:c r="C40" s="22"/>
       <x:c r="D40" s="24"/>
       <x:c r="E40" s="24"/>
       <x:c r="F40" s="20"/>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" s="20"/>
-      <x:c r="B41" s="20"/>
+      <x:c r="A41" s="32"/>
+      <x:c r="B41" s="32"/>
       <x:c r="C41" s="22"/>
       <x:c r="D41" s="24"/>
       <x:c r="E41" s="24"/>
       <x:c r="F41" s="20"/>
     </x:row>
     <x:row r="42">
-      <x:c r="A42" s="20"/>
-      <x:c r="B42" s="20"/>
+      <x:c r="A42" s="32"/>
+      <x:c r="B42" s="32"/>
       <x:c r="C42" s="22"/>
       <x:c r="D42" s="24"/>
       <x:c r="E42" s="24"/>
       <x:c r="F42" s="20"/>
     </x:row>
     <x:row r="43">
-      <x:c r="A43" s="20"/>
-      <x:c r="B43" s="20"/>
+      <x:c r="A43" s="32"/>
+      <x:c r="B43" s="32"/>
       <x:c r="C43" s="22"/>
       <x:c r="D43" s="24"/>
       <x:c r="E43" s="24"/>
       <x:c r="F43" s="20"/>
     </x:row>
     <x:row r="44">
-      <x:c r="A44" s="20"/>
-      <x:c r="B44" s="20"/>
+      <x:c r="A44" s="32"/>
+      <x:c r="B44" s="32"/>
       <x:c r="C44" s="22"/>
       <x:c r="D44" s="24"/>
       <x:c r="E44" s="24"/>
       <x:c r="F44" s="20"/>
     </x:row>
     <x:row r="45">
-      <x:c r="A45" s="20"/>
-      <x:c r="B45" s="20"/>
+      <x:c r="A45" s="32"/>
+      <x:c r="B45" s="32"/>
       <x:c r="C45" s="22"/>
       <x:c r="D45" s="24"/>
       <x:c r="E45" s="24"/>
       <x:c r="F45" s="20"/>
     </x:row>
     <x:row r="46">
-      <x:c r="A46" s="20"/>
-      <x:c r="B46" s="20"/>
+      <x:c r="A46" s="32"/>
+      <x:c r="B46" s="32"/>
       <x:c r="C46" s="22"/>
       <x:c r="D46" s="24"/>
       <x:c r="E46" s="24"/>
       <x:c r="F46" s="20"/>
     </x:row>
     <x:row r="47">
-      <x:c r="A47" s="20"/>
-      <x:c r="B47" s="20"/>
+      <x:c r="A47" s="32"/>
+      <x:c r="B47" s="32"/>
       <x:c r="C47" s="22"/>
       <x:c r="D47" s="24"/>
       <x:c r="E47" s="24"/>
       <x:c r="F47" s="20"/>
     </x:row>
     <x:row r="48">
-      <x:c r="A48" s="20"/>
-      <x:c r="B48" s="20"/>
+      <x:c r="A48" s="32"/>
+      <x:c r="B48" s="32"/>
       <x:c r="C48" s="22"/>
       <x:c r="D48" s="24"/>
       <x:c r="E48" s="24"/>
       <x:c r="F48" s="20"/>
     </x:row>
     <x:row r="49">
-      <x:c r="A49" s="20"/>
-      <x:c r="B49" s="20"/>
+      <x:c r="A49" s="32"/>
+      <x:c r="B49" s="32"/>
       <x:c r="C49" s="22"/>
       <x:c r="D49" s="24"/>
       <x:c r="E49" s="24"/>
       <x:c r="F49" s="20"/>
     </x:row>
     <x:row r="50">
-      <x:c r="A50" s="20"/>
-      <x:c r="B50" s="20"/>
+      <x:c r="A50" s="32"/>
+      <x:c r="B50" s="32"/>
       <x:c r="C50" s="22"/>
       <x:c r="D50" s="24"/>
       <x:c r="E50" s="24"/>
       <x:c r="F50" s="20"/>
     </x:row>
     <x:row r="51">
-      <x:c r="A51" s="20"/>
-      <x:c r="B51" s="20"/>
+      <x:c r="A51" s="32"/>
+      <x:c r="B51" s="32"/>
       <x:c r="C51" s="22"/>
       <x:c r="D51" s="24"/>
       <x:c r="E51" s="24"/>
       <x:c r="F51" s="20"/>
     </x:row>
     <x:row r="52">
-      <x:c r="A52" s="20"/>
-      <x:c r="B52" s="20"/>
+      <x:c r="A52" s="32"/>
+      <x:c r="B52" s="32"/>
       <x:c r="C52" s="22"/>
       <x:c r="D52" s="24"/>
       <x:c r="E52" s="24"/>
       <x:c r="F52" s="20"/>
     </x:row>
     <x:row r="53">
-      <x:c r="A53" s="20"/>
-      <x:c r="B53" s="20"/>
+      <x:c r="A53" s="32"/>
+      <x:c r="B53" s="32"/>
       <x:c r="C53" s="22"/>
       <x:c r="D53" s="24"/>
       <x:c r="E53" s="24"/>
       <x:c r="F53" s="20"/>
     </x:row>
     <x:row r="54">
-      <x:c r="A54" s="20"/>
-      <x:c r="B54" s="20"/>
+      <x:c r="A54" s="32"/>
+      <x:c r="B54" s="32"/>
       <x:c r="C54" s="22"/>
       <x:c r="D54" s="24"/>
       <x:c r="E54" s="24"/>
       <x:c r="F54" s="20"/>
     </x:row>
     <x:row r="55">
-      <x:c r="A55" s="20"/>
-      <x:c r="B55" s="20"/>
+      <x:c r="A55" s="32"/>
+      <x:c r="B55" s="32"/>
       <x:c r="C55" s="22"/>
       <x:c r="D55" s="24"/>
       <x:c r="E55" s="24"/>
       <x:c r="F55" s="20"/>
     </x:row>
     <x:row r="56">
-      <x:c r="A56" s="20"/>
-      <x:c r="B56" s="20"/>
+      <x:c r="A56" s="32"/>
+      <x:c r="B56" s="32"/>
       <x:c r="C56" s="22"/>
       <x:c r="D56" s="24"/>
       <x:c r="E56" s="24"/>

</xml_diff>